<commit_message>
Add accordion-faq, business-goal, plan-comparison blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (16):
- blocks/accordion-faq/_accordion-faq.json
- blocks/business-goal/_business-goal.json
- blocks/plan-comparison/_plan-comparison.json
- blocks/plan-comparison/plan-comparison.css
- blocks/plan-comparison/plan-comparison.js
- component-definition.json
- component-filters.json
- component-models.json
- models/_section.json
- tools/importer/import-product-page.bundle.js
- tools/importer/import-product-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/plan-comparison.js
- tools/importer/reports/import-product-page.report.xlsx
- tools/importer/reports/products/wireless-plans.report.json
- tools/importer/urls-single.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-product-page.report.xlsx
+++ b/tools/importer/reports/import-product-page.report.xlsx
@@ -466,13 +466,13 @@
     <t>products/wireless-plans.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-product","cards-product","cards-product","cards-value","cards-value","hero-dark","hero-dark","hero-dark","columns-offer","accordion-faq"]</t>
+    <t>["hero-banner","cards-product","cards-product","cards-product","cards-value","cards-value","hero-dark","hero-dark","hero-dark","columns-offer","accordion-faq","plan-comparison"]</t>
   </si>
   <si>
     <t>products/wireless-plans</t>
   </si>
   <si>
-    <t>2026-03-02T13:40:12.511Z</t>
+    <t>2026-03-02T14:53:49.922Z</t>
   </si>
   <si>
     <t>Business Cell Phone Plans | AT&amp;T Business Wireless &amp; Mobile</t>

</xml_diff>